<commit_message>
project setup wizard updated.
</commit_message>
<xml_diff>
--- a/backend/_data_list/house_list_master.xlsx
+++ b/backend/_data_list/house_list_master.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\Telegram_Project\OrangeFlow_Dev\_data_list\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\Telegram_Project\Orange-Flow-Next-Js\backend\_data_list\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{22FDA2CB-AB0C-4D10-9688-25989C9996D3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{76D97AA0-4929-404A-B61E-E42271C004F4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="14430" yWindow="0" windowWidth="14475" windowHeight="15585" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -178,7 +178,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="165" formatCode="[$-409]d/mmm/yy;@"/>
+    <numFmt numFmtId="164" formatCode="[$-409]d/mmm/yy;@"/>
   </numFmts>
   <fonts count="2" x14ac:knownFonts="1">
     <font>
@@ -220,7 +220,7 @@
   </cellStyleXfs>
   <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
   </cellXfs>
   <cellStyles count="2">

</xml_diff>